<commit_message>
added temperature and drink type
</commit_message>
<xml_diff>
--- a/labeled/Hydrocare_ffinal.xlsx
+++ b/labeled/Hydrocare_ffinal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alireza.mohammadshafie/Documents/hydrocare/labeled/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE63D1F-E9F7-A04B-A5C9-9D9924559CDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D96F8C8-9C03-2046-8671-2BFBED2F5D34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="52">
   <si>
     <t>ID</t>
   </si>
@@ -149,6 +149,33 @@
   </si>
   <si>
     <t>d</t>
+  </si>
+  <si>
+    <t>drink</t>
+  </si>
+  <si>
+    <t>temp</t>
+  </si>
+  <si>
+    <t>coffee</t>
+  </si>
+  <si>
+    <t>coke-r</t>
+  </si>
+  <si>
+    <t>coke-z</t>
+  </si>
+  <si>
+    <t>water</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>n</t>
   </si>
 </sst>
 </file>
@@ -516,17 +543,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA57"/>
+  <dimension ref="A1:AC57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="14.6640625" customWidth="1"/>
     <col min="4" max="4" width="12.5" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" customWidth="1"/>
-    <col min="9" max="9" width="24.1640625" customWidth="1"/>
-    <col min="10" max="10" width="22.1640625" customWidth="1"/>
+    <col min="5" max="7" width="17.33203125" customWidth="1"/>
+    <col min="8" max="8" width="33.33203125" customWidth="1"/>
+    <col min="11" max="11" width="24.1640625" customWidth="1"/>
+    <col min="12" max="12" width="22.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -543,73 +571,79 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1">
+      <c r="P1" s="1">
         <v>5</v>
       </c>
-      <c r="O1" s="1">
+      <c r="Q1" s="1">
         <v>6</v>
       </c>
-      <c r="P1" s="1">
+      <c r="R1" s="1">
         <v>7</v>
       </c>
-      <c r="Q1" s="1">
+      <c r="S1" s="1">
         <v>8</v>
       </c>
-      <c r="R1" s="1">
+      <c r="T1" s="1">
         <v>9</v>
       </c>
-      <c r="S1" s="1">
+      <c r="U1" s="1">
         <v>10</v>
       </c>
-      <c r="T1" s="1">
+      <c r="V1" s="1">
         <v>11</v>
       </c>
-      <c r="U1" s="1">
+      <c r="W1" s="1">
         <v>12</v>
       </c>
-      <c r="V1" s="1">
+      <c r="X1" s="1">
         <v>13</v>
       </c>
-      <c r="W1" s="1">
+      <c r="Y1" s="1">
         <v>14</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>6</v>
       </c>
@@ -626,34 +660,40 @@
         <v>540.4</v>
       </c>
       <c r="F2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H2" t="s">
         <v>24</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>39</v>
       </c>
-      <c r="I2">
+      <c r="K2">
         <v>538.6</v>
       </c>
-      <c r="J2">
+      <c r="L2">
         <v>465.2</v>
       </c>
-      <c r="K2">
+      <c r="M2">
         <v>404.3</v>
       </c>
-      <c r="L2">
+      <c r="N2">
         <v>339.3</v>
       </c>
-      <c r="M2">
+      <c r="O2">
         <v>267</v>
       </c>
-      <c r="N2">
+      <c r="P2">
         <v>220.2</v>
       </c>
-      <c r="O2">
+      <c r="Q2">
         <v>190.9</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>7</v>
       </c>
@@ -670,37 +710,43 @@
         <v>272.60000000000002</v>
       </c>
       <c r="F3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H3" t="s">
         <v>25</v>
       </c>
-      <c r="H3" t="s">
+      <c r="J3" t="s">
         <v>39</v>
       </c>
-      <c r="I3">
+      <c r="K3">
         <v>272.60000000000002</v>
       </c>
-      <c r="J3">
+      <c r="L3">
         <v>261</v>
       </c>
-      <c r="K3">
+      <c r="M3">
         <v>246.7</v>
       </c>
-      <c r="L3">
+      <c r="N3">
         <v>234.1</v>
       </c>
-      <c r="M3">
+      <c r="O3">
         <v>221.5</v>
       </c>
-      <c r="N3">
+      <c r="P3">
         <v>210.3</v>
       </c>
-      <c r="O3">
+      <c r="Q3">
         <v>190.5</v>
       </c>
-      <c r="P3">
+      <c r="R3">
         <v>173.4</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>8</v>
       </c>
@@ -717,34 +763,40 @@
         <v>542.6</v>
       </c>
       <c r="F4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" t="s">
         <v>26</v>
       </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>39</v>
       </c>
-      <c r="I4">
+      <c r="K4">
         <v>540.6</v>
       </c>
-      <c r="J4">
+      <c r="L4">
         <v>524.79999999999995</v>
       </c>
-      <c r="K4">
+      <c r="M4">
         <v>501.6</v>
       </c>
-      <c r="L4">
+      <c r="N4">
         <v>480.1</v>
       </c>
-      <c r="M4">
+      <c r="O4">
         <v>470.5</v>
       </c>
-      <c r="N4">
+      <c r="P4">
         <v>459.5</v>
       </c>
-      <c r="O4">
+      <c r="Q4">
         <v>450.7</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>9</v>
       </c>
@@ -761,37 +813,43 @@
         <v>542.9</v>
       </c>
       <c r="F5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" t="s">
+        <v>46</v>
+      </c>
+      <c r="H5" t="s">
         <v>26</v>
       </c>
-      <c r="H5" t="s">
+      <c r="J5" t="s">
         <v>40</v>
       </c>
-      <c r="I5">
+      <c r="K5">
         <v>540.79999999999995</v>
       </c>
-      <c r="J5">
+      <c r="L5">
         <v>531.70000000000005</v>
       </c>
-      <c r="K5">
+      <c r="M5">
         <v>519.29999999999995</v>
       </c>
-      <c r="L5">
+      <c r="N5">
         <v>507.9</v>
       </c>
-      <c r="M5">
+      <c r="O5">
         <v>493.9</v>
       </c>
-      <c r="N5">
+      <c r="P5">
         <v>480</v>
       </c>
-      <c r="O5">
+      <c r="Q5">
         <v>465.3</v>
       </c>
-      <c r="P5">
+      <c r="R5">
         <v>449.9</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>10</v>
       </c>
@@ -808,40 +866,46 @@
         <v>521.70000000000005</v>
       </c>
       <c r="F6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" t="s">
         <v>27</v>
       </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>39</v>
       </c>
-      <c r="I6">
+      <c r="K6">
         <v>518.79999999999995</v>
       </c>
-      <c r="J6">
+      <c r="L6">
         <v>516.1</v>
       </c>
-      <c r="K6">
+      <c r="M6">
         <v>512.1</v>
       </c>
-      <c r="L6">
+      <c r="N6">
         <v>510.3</v>
       </c>
-      <c r="M6">
+      <c r="O6">
         <v>506.8</v>
       </c>
-      <c r="N6">
+      <c r="P6">
         <v>504.7</v>
       </c>
-      <c r="O6">
+      <c r="Q6">
         <v>498.9</v>
       </c>
-      <c r="P6">
+      <c r="R6">
         <v>497.2</v>
       </c>
-      <c r="Q6">
+      <c r="S6">
         <v>494.2</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>11</v>
       </c>
@@ -858,40 +922,46 @@
         <v>228.4</v>
       </c>
       <c r="F7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H7" t="s">
         <v>28</v>
       </c>
-      <c r="H7" t="s">
+      <c r="J7" t="s">
         <v>39</v>
       </c>
-      <c r="I7">
+      <c r="K7">
         <v>228.4</v>
       </c>
-      <c r="J7">
+      <c r="L7">
         <v>219.3</v>
       </c>
-      <c r="K7">
+      <c r="M7">
         <v>198.8</v>
       </c>
-      <c r="L7">
+      <c r="N7">
         <v>179.9</v>
       </c>
-      <c r="M7">
+      <c r="O7">
         <v>139.80000000000001</v>
       </c>
-      <c r="N7">
+      <c r="P7">
         <v>126.7</v>
       </c>
-      <c r="O7">
+      <c r="Q7">
         <v>120</v>
       </c>
-      <c r="P7">
+      <c r="R7">
         <v>97.3</v>
       </c>
-      <c r="Q7">
+      <c r="S7">
         <v>75.3</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>12</v>
       </c>
@@ -908,49 +978,55 @@
         <v>519.4</v>
       </c>
       <c r="F8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" t="s">
         <v>29</v>
       </c>
-      <c r="H8" t="s">
+      <c r="J8" t="s">
         <v>40</v>
       </c>
-      <c r="I8">
+      <c r="K8">
         <v>519.20000000000005</v>
       </c>
-      <c r="J8">
+      <c r="L8">
         <v>478.2</v>
       </c>
-      <c r="K8">
+      <c r="M8">
         <v>424.4</v>
       </c>
-      <c r="L8">
+      <c r="N8">
         <v>363</v>
       </c>
-      <c r="M8">
+      <c r="O8">
         <v>316.2</v>
       </c>
-      <c r="N8">
+      <c r="P8">
         <v>255.2</v>
       </c>
-      <c r="O8">
+      <c r="Q8">
         <v>204.8</v>
       </c>
-      <c r="P8">
+      <c r="R8">
         <v>160</v>
       </c>
-      <c r="Q8">
+      <c r="S8">
         <v>101.6</v>
       </c>
-      <c r="R8">
+      <c r="T8">
         <v>62.6</v>
       </c>
-      <c r="S8">
+      <c r="U8">
         <v>24.2</v>
       </c>
-      <c r="T8">
+      <c r="V8">
         <v>11.5</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>13</v>
       </c>
@@ -967,52 +1043,58 @@
         <v>521.20000000000005</v>
       </c>
       <c r="F9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" t="s">
         <v>30</v>
       </c>
-      <c r="H9" t="s">
+      <c r="J9" t="s">
         <v>39</v>
       </c>
-      <c r="I9">
+      <c r="K9">
         <v>519.29999999999995</v>
       </c>
-      <c r="J9">
+      <c r="L9">
         <v>492.7</v>
       </c>
-      <c r="K9">
+      <c r="M9">
         <v>471.9</v>
       </c>
-      <c r="L9">
+      <c r="N9">
         <v>450.8</v>
       </c>
-      <c r="M9">
+      <c r="O9">
         <v>431</v>
       </c>
-      <c r="N9">
+      <c r="P9">
         <v>410.4</v>
       </c>
-      <c r="O9">
+      <c r="Q9">
         <v>388.4</v>
       </c>
-      <c r="P9">
+      <c r="R9">
         <v>366.4</v>
       </c>
-      <c r="Q9">
+      <c r="S9">
         <v>345.5</v>
       </c>
-      <c r="R9">
+      <c r="T9">
         <v>323.2</v>
       </c>
-      <c r="S9">
+      <c r="U9">
         <v>302.5</v>
       </c>
-      <c r="T9">
+      <c r="V9">
         <v>283.60000000000002</v>
       </c>
-      <c r="U9">
+      <c r="W9">
         <v>269.10000000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>14</v>
       </c>
@@ -1029,46 +1111,52 @@
         <v>515.9</v>
       </c>
       <c r="F10" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" t="s">
         <v>29</v>
       </c>
-      <c r="H10" t="s">
+      <c r="J10" t="s">
         <v>39</v>
       </c>
-      <c r="I10">
+      <c r="K10">
         <v>515.20000000000005</v>
       </c>
-      <c r="J10">
+      <c r="L10">
         <v>427.4</v>
       </c>
-      <c r="K10">
+      <c r="M10">
         <v>374.2</v>
       </c>
-      <c r="L10">
+      <c r="N10">
         <v>330.4</v>
       </c>
-      <c r="M10">
+      <c r="O10">
         <v>291.3</v>
       </c>
-      <c r="N10">
+      <c r="P10">
         <v>255</v>
       </c>
-      <c r="O10">
+      <c r="Q10">
         <v>221.2</v>
       </c>
-      <c r="P10">
+      <c r="R10">
         <v>166.9</v>
       </c>
-      <c r="Q10">
+      <c r="S10">
         <v>108.2</v>
       </c>
-      <c r="R10">
+      <c r="T10">
         <v>49.5</v>
       </c>
-      <c r="S10">
+      <c r="U10">
         <v>9.5</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>15</v>
       </c>
@@ -1085,37 +1173,43 @@
         <v>547.20000000000005</v>
       </c>
       <c r="F11" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" t="s">
         <v>31</v>
       </c>
-      <c r="H11" t="s">
+      <c r="J11" t="s">
         <v>40</v>
       </c>
-      <c r="I11">
+      <c r="K11">
         <v>545.70000000000005</v>
       </c>
-      <c r="J11">
+      <c r="L11">
         <v>533.79999999999995</v>
       </c>
-      <c r="K11">
+      <c r="M11">
         <v>516.4</v>
       </c>
-      <c r="L11">
+      <c r="N11">
         <v>497.3</v>
       </c>
-      <c r="M11">
+      <c r="O11">
         <v>475</v>
       </c>
-      <c r="N11">
+      <c r="P11">
         <v>455.6</v>
       </c>
-      <c r="O11">
+      <c r="Q11">
         <v>430.9</v>
       </c>
-      <c r="P11">
+      <c r="R11">
         <v>414.2</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>16</v>
       </c>
@@ -1132,58 +1226,64 @@
         <v>295.10000000000002</v>
       </c>
       <c r="F12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G12" t="s">
+        <v>45</v>
+      </c>
+      <c r="H12" t="s">
         <v>25</v>
       </c>
-      <c r="H12" t="s">
+      <c r="J12" t="s">
         <v>39</v>
       </c>
-      <c r="I12">
+      <c r="K12">
         <v>289.5</v>
       </c>
-      <c r="J12">
+      <c r="L12">
         <v>279.89999999999998</v>
       </c>
-      <c r="K12">
+      <c r="M12">
         <v>265.60000000000002</v>
       </c>
-      <c r="L12">
+      <c r="N12">
         <v>251.2</v>
       </c>
-      <c r="M12">
+      <c r="O12">
         <v>236.4</v>
       </c>
-      <c r="N12">
+      <c r="P12">
         <v>221.1</v>
       </c>
-      <c r="O12">
+      <c r="Q12">
         <v>205.4</v>
       </c>
-      <c r="P12">
+      <c r="R12">
         <v>192.5</v>
       </c>
-      <c r="Q12">
+      <c r="S12">
         <v>181.6</v>
       </c>
-      <c r="R12">
+      <c r="T12">
         <v>171</v>
       </c>
-      <c r="S12">
+      <c r="U12">
         <v>159.30000000000001</v>
       </c>
-      <c r="T12">
+      <c r="V12">
         <v>146.6</v>
       </c>
-      <c r="U12">
+      <c r="W12">
         <v>136.80000000000001</v>
       </c>
-      <c r="V12">
+      <c r="X12">
         <v>127.5</v>
       </c>
-      <c r="W12">
+      <c r="Y12">
         <v>117.6</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>17</v>
       </c>
@@ -1200,43 +1300,49 @@
         <v>542</v>
       </c>
       <c r="F13" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" t="s">
+        <v>46</v>
+      </c>
+      <c r="H13" t="s">
         <v>24</v>
       </c>
-      <c r="H13" t="s">
+      <c r="J13" t="s">
         <v>39</v>
       </c>
-      <c r="I13">
+      <c r="K13">
         <v>539.79999999999995</v>
       </c>
-      <c r="J13">
+      <c r="L13">
         <v>514</v>
       </c>
-      <c r="K13">
+      <c r="M13">
         <v>490.8</v>
       </c>
-      <c r="L13">
+      <c r="N13">
         <v>479</v>
       </c>
-      <c r="M13">
+      <c r="O13">
         <v>468.7</v>
       </c>
-      <c r="N13">
+      <c r="P13">
         <v>450</v>
       </c>
-      <c r="O13">
+      <c r="Q13">
         <v>432.8</v>
       </c>
-      <c r="P13">
+      <c r="R13">
         <v>408.4</v>
       </c>
-      <c r="Q13">
+      <c r="S13">
         <v>388.4</v>
       </c>
-      <c r="R13">
+      <c r="T13">
         <v>366.9</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>18</v>
       </c>
@@ -1253,58 +1359,64 @@
         <v>543.29999999999995</v>
       </c>
       <c r="F14" t="s">
+        <v>49</v>
+      </c>
+      <c r="G14" t="s">
+        <v>46</v>
+      </c>
+      <c r="H14" t="s">
         <v>24</v>
       </c>
-      <c r="H14" t="s">
+      <c r="J14" t="s">
         <v>40</v>
       </c>
-      <c r="I14">
+      <c r="K14">
         <v>541.6</v>
       </c>
-      <c r="J14">
+      <c r="L14">
         <v>517.6</v>
       </c>
-      <c r="K14">
+      <c r="M14">
         <v>504.7</v>
       </c>
-      <c r="L14">
+      <c r="N14">
         <v>493.7</v>
       </c>
-      <c r="M14">
+      <c r="O14">
         <v>480.4</v>
       </c>
-      <c r="N14">
+      <c r="P14">
         <v>468.2</v>
       </c>
-      <c r="O14">
+      <c r="Q14">
         <v>456.5</v>
       </c>
-      <c r="P14">
+      <c r="R14">
         <v>444.2</v>
       </c>
-      <c r="Q14">
+      <c r="S14">
         <v>431.9</v>
       </c>
-      <c r="R14">
+      <c r="T14">
         <v>420.6</v>
       </c>
-      <c r="S14">
+      <c r="U14">
         <v>409.6</v>
       </c>
-      <c r="T14">
+      <c r="V14">
         <v>398.8</v>
       </c>
-      <c r="U14">
+      <c r="W14">
         <v>387</v>
       </c>
-      <c r="V14">
+      <c r="X14">
         <v>377.6</v>
       </c>
-      <c r="W14">
+      <c r="Y14">
         <v>365.3</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>19</v>
       </c>
@@ -1321,28 +1433,34 @@
         <v>518</v>
       </c>
       <c r="F15" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" t="s">
+        <v>47</v>
+      </c>
+      <c r="H15" t="s">
         <v>30</v>
       </c>
-      <c r="H15" t="s">
+      <c r="J15" t="s">
         <v>39</v>
       </c>
-      <c r="I15">
+      <c r="K15">
         <v>472.9</v>
       </c>
-      <c r="J15">
+      <c r="L15">
         <v>410.8</v>
       </c>
-      <c r="K15">
+      <c r="M15">
         <v>339.7</v>
       </c>
-      <c r="L15">
+      <c r="N15">
         <v>275.2</v>
       </c>
-      <c r="M15">
+      <c r="O15">
         <v>204</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>20</v>
       </c>
@@ -1356,40 +1474,46 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" t="s">
+        <v>48</v>
+      </c>
+      <c r="H16" t="s">
         <v>29</v>
       </c>
-      <c r="H16" t="s">
+      <c r="J16" t="s">
         <v>39</v>
       </c>
-      <c r="I16">
+      <c r="K16">
         <v>485.4</v>
       </c>
-      <c r="J16">
+      <c r="L16">
         <v>411.9</v>
       </c>
-      <c r="K16">
+      <c r="M16">
         <v>352.9</v>
       </c>
-      <c r="L16">
+      <c r="N16">
         <v>293.5</v>
       </c>
-      <c r="M16">
+      <c r="O16">
         <v>238.2</v>
       </c>
-      <c r="N16">
+      <c r="P16">
         <v>180.2</v>
       </c>
-      <c r="O16">
+      <c r="Q16">
         <v>120.5</v>
       </c>
-      <c r="P16">
+      <c r="R16">
         <v>63.4</v>
       </c>
-      <c r="Q16">
+      <c r="S16">
         <v>8.5</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>21</v>
       </c>
@@ -1406,37 +1530,43 @@
         <v>262.7</v>
       </c>
       <c r="F17" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" t="s">
+        <v>45</v>
+      </c>
+      <c r="H17" t="s">
         <v>32</v>
       </c>
-      <c r="H17" t="s">
+      <c r="J17" t="s">
         <v>39</v>
       </c>
-      <c r="I17">
+      <c r="K17">
         <v>262.60000000000002</v>
       </c>
-      <c r="J17">
+      <c r="L17">
         <v>246.9</v>
       </c>
-      <c r="K17">
+      <c r="M17">
         <v>214.4</v>
       </c>
-      <c r="L17">
+      <c r="N17">
         <v>193.4</v>
       </c>
-      <c r="M17">
+      <c r="O17">
         <v>159.5</v>
       </c>
-      <c r="N17">
+      <c r="P17">
         <v>136.4</v>
       </c>
-      <c r="O17">
+      <c r="Q17">
         <v>115.9</v>
       </c>
-      <c r="P17">
+      <c r="R17">
         <v>97.4</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>22</v>
       </c>
@@ -1453,49 +1583,55 @@
         <v>280.3</v>
       </c>
       <c r="F18" t="s">
+        <v>50</v>
+      </c>
+      <c r="G18" t="s">
+        <v>45</v>
+      </c>
+      <c r="H18" t="s">
         <v>25</v>
       </c>
-      <c r="H18" t="s">
+      <c r="J18" t="s">
         <v>39</v>
       </c>
-      <c r="I18">
+      <c r="K18">
         <v>292.2</v>
       </c>
-      <c r="J18">
+      <c r="L18">
         <v>281.2</v>
       </c>
-      <c r="K18">
+      <c r="M18">
         <v>269.39999999999998</v>
       </c>
-      <c r="L18">
+      <c r="N18">
         <v>256.60000000000002</v>
       </c>
-      <c r="M18">
+      <c r="O18">
         <v>239.9</v>
       </c>
-      <c r="N18">
+      <c r="P18">
         <v>222.5</v>
       </c>
-      <c r="O18">
+      <c r="Q18">
         <v>201.8</v>
       </c>
-      <c r="P18">
+      <c r="R18">
         <v>180.4</v>
       </c>
-      <c r="Q18">
+      <c r="S18">
         <v>165.7</v>
       </c>
-      <c r="R18">
+      <c r="T18">
         <v>145.19999999999999</v>
       </c>
-      <c r="S18">
+      <c r="U18">
         <v>126.1</v>
       </c>
-      <c r="T18">
+      <c r="V18">
         <v>105.5</v>
       </c>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>23</v>
       </c>
@@ -1509,40 +1645,46 @@
         <v>1.05</v>
       </c>
       <c r="F19" t="s">
+        <v>49</v>
+      </c>
+      <c r="G19" t="s">
+        <v>46</v>
+      </c>
+      <c r="H19" t="s">
         <v>24</v>
       </c>
-      <c r="H19" t="s">
+      <c r="J19" t="s">
         <v>39</v>
       </c>
-      <c r="I19">
+      <c r="K19">
         <v>544.70000000000005</v>
       </c>
-      <c r="J19">
+      <c r="L19">
         <v>470.7</v>
       </c>
-      <c r="K19">
+      <c r="M19">
         <v>422.6</v>
       </c>
-      <c r="L19">
+      <c r="N19">
         <v>350.9</v>
       </c>
-      <c r="M19">
+      <c r="O19">
         <v>287.89999999999998</v>
       </c>
-      <c r="N19">
+      <c r="P19">
         <v>221.7</v>
       </c>
-      <c r="O19">
+      <c r="Q19">
         <v>156.5</v>
       </c>
-      <c r="P19">
+      <c r="R19">
         <v>99.1</v>
       </c>
-      <c r="Q19">
+      <c r="S19">
         <v>21.1</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>24</v>
       </c>
@@ -1559,46 +1701,52 @@
         <v>518.9</v>
       </c>
       <c r="F20" t="s">
+        <v>49</v>
+      </c>
+      <c r="G20" t="s">
+        <v>47</v>
+      </c>
+      <c r="H20" t="s">
         <v>33</v>
       </c>
-      <c r="H20" t="s">
+      <c r="J20" t="s">
         <v>39</v>
       </c>
-      <c r="I20">
+      <c r="K20">
         <v>517</v>
       </c>
-      <c r="J20">
+      <c r="L20">
         <v>497.5</v>
       </c>
-      <c r="K20">
+      <c r="M20">
         <v>468.7</v>
       </c>
-      <c r="L20">
+      <c r="N20">
         <v>445.1</v>
       </c>
-      <c r="M20">
+      <c r="O20">
         <v>422.3</v>
       </c>
-      <c r="N20">
+      <c r="P20">
         <v>400.8</v>
       </c>
-      <c r="O20">
+      <c r="Q20">
         <v>394.6</v>
       </c>
-      <c r="P20">
+      <c r="R20">
         <v>381.8</v>
       </c>
-      <c r="Q20">
+      <c r="S20">
         <v>369.9</v>
       </c>
-      <c r="R20">
+      <c r="T20">
         <v>361.5</v>
       </c>
-      <c r="S20">
+      <c r="U20">
         <v>354.7</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>26</v>
       </c>
@@ -1615,31 +1763,37 @@
         <v>523.70000000000005</v>
       </c>
       <c r="F21" t="s">
+        <v>49</v>
+      </c>
+      <c r="G21" t="s">
+        <v>47</v>
+      </c>
+      <c r="H21" t="s">
         <v>30</v>
       </c>
-      <c r="H21" t="s">
+      <c r="J21" t="s">
         <v>39</v>
       </c>
-      <c r="I21">
+      <c r="K21">
         <v>521.5</v>
       </c>
-      <c r="J21">
+      <c r="L21">
         <v>486.4</v>
       </c>
-      <c r="K21">
+      <c r="M21">
         <v>468.5</v>
       </c>
-      <c r="L21">
+      <c r="N21">
         <v>454.5</v>
       </c>
-      <c r="M21">
+      <c r="O21">
         <v>444.9</v>
       </c>
-      <c r="N21">
+      <c r="P21">
         <v>434.7</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>27</v>
       </c>
@@ -1656,31 +1810,37 @@
         <v>516.1</v>
       </c>
       <c r="F22" t="s">
+        <v>51</v>
+      </c>
+      <c r="G22" t="s">
+        <v>48</v>
+      </c>
+      <c r="H22" t="s">
         <v>29</v>
       </c>
-      <c r="H22" t="s">
+      <c r="J22" t="s">
         <v>39</v>
       </c>
-      <c r="I22">
+      <c r="K22">
         <v>515.4</v>
       </c>
-      <c r="J22">
+      <c r="L22">
         <v>411.6</v>
       </c>
-      <c r="K22">
+      <c r="M22">
         <v>320.10000000000002</v>
       </c>
-      <c r="L22">
+      <c r="N22">
         <v>188.4</v>
       </c>
-      <c r="M22">
+      <c r="O22">
         <v>95.5</v>
       </c>
-      <c r="N22">
+      <c r="P22">
         <v>9.8000000000000007</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>28</v>
       </c>
@@ -1697,43 +1857,49 @@
         <v>201.8</v>
       </c>
       <c r="F23" t="s">
+        <v>49</v>
+      </c>
+      <c r="G23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H23" t="s">
         <v>34</v>
       </c>
-      <c r="H23" t="s">
+      <c r="J23" t="s">
         <v>39</v>
       </c>
-      <c r="I23">
+      <c r="K23">
         <v>201.8</v>
       </c>
-      <c r="J23">
+      <c r="L23">
         <v>188</v>
       </c>
-      <c r="K23">
+      <c r="M23">
         <v>177</v>
       </c>
-      <c r="L23">
+      <c r="N23">
         <v>161.6</v>
       </c>
-      <c r="M23">
+      <c r="O23">
         <v>138.19999999999999</v>
       </c>
-      <c r="N23">
+      <c r="P23">
         <v>126.3</v>
       </c>
-      <c r="O23">
+      <c r="Q23">
         <v>101.4</v>
       </c>
-      <c r="P23">
+      <c r="R23">
         <v>87.8</v>
       </c>
-      <c r="Q23">
+      <c r="S23">
         <v>50.8</v>
       </c>
-      <c r="R23">
+      <c r="T23">
         <v>21.8</v>
       </c>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>29</v>
       </c>
@@ -1750,43 +1916,49 @@
         <v>330.5</v>
       </c>
       <c r="F24" t="s">
+        <v>49</v>
+      </c>
+      <c r="G24" t="s">
+        <v>47</v>
+      </c>
+      <c r="H24" t="s">
         <v>34</v>
       </c>
-      <c r="H24" t="s">
+      <c r="J24" t="s">
         <v>40</v>
       </c>
-      <c r="I24">
+      <c r="K24">
         <v>331.2</v>
       </c>
-      <c r="J24">
+      <c r="L24">
         <v>316.7</v>
       </c>
-      <c r="K24">
+      <c r="M24">
         <v>303.7</v>
       </c>
-      <c r="L24">
+      <c r="N24">
         <v>286.10000000000002</v>
       </c>
-      <c r="M24">
+      <c r="O24">
         <v>265.5</v>
       </c>
-      <c r="N24">
+      <c r="P24">
         <v>249.7</v>
       </c>
-      <c r="O24">
+      <c r="Q24">
         <v>236.2</v>
       </c>
-      <c r="P24">
+      <c r="R24">
         <v>226.7</v>
       </c>
-      <c r="Q24">
+      <c r="S24">
         <v>212</v>
       </c>
-      <c r="R24">
+      <c r="T24">
         <v>204.1</v>
       </c>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>30</v>
       </c>
@@ -1803,58 +1975,64 @@
         <v>548.79999999999995</v>
       </c>
       <c r="F25" t="s">
+        <v>49</v>
+      </c>
+      <c r="G25" t="s">
+        <v>46</v>
+      </c>
+      <c r="H25" t="s">
         <v>24</v>
       </c>
-      <c r="H25" t="s">
+      <c r="J25" t="s">
         <v>39</v>
       </c>
-      <c r="I25">
+      <c r="K25">
         <v>546.6</v>
       </c>
-      <c r="J25">
+      <c r="L25">
         <v>532.5</v>
       </c>
-      <c r="K25">
+      <c r="M25">
         <v>490</v>
       </c>
-      <c r="L25">
+      <c r="N25">
         <v>464.6</v>
       </c>
-      <c r="M25">
+      <c r="O25">
         <v>437.8</v>
       </c>
-      <c r="N25">
+      <c r="P25">
         <v>416.4</v>
       </c>
-      <c r="O25">
+      <c r="Q25">
         <v>407</v>
       </c>
-      <c r="P25">
+      <c r="R25">
         <v>387.6</v>
       </c>
-      <c r="Q25">
+      <c r="S25">
         <v>375.6</v>
       </c>
-      <c r="R25">
+      <c r="T25">
         <v>352.9</v>
       </c>
-      <c r="S25">
+      <c r="U25">
         <v>339.9</v>
       </c>
-      <c r="T25">
+      <c r="V25">
         <v>330.4</v>
       </c>
-      <c r="U25">
+      <c r="W25">
         <v>304.89999999999998</v>
       </c>
-      <c r="V25">
+      <c r="X25">
         <v>288.3</v>
       </c>
-      <c r="W25">
+      <c r="Y25">
         <v>266.39999999999998</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>31</v>
       </c>
@@ -1871,37 +2049,43 @@
         <v>592.5</v>
       </c>
       <c r="F26" t="s">
+        <v>51</v>
+      </c>
+      <c r="G26" t="s">
+        <v>48</v>
+      </c>
+      <c r="H26" t="s">
         <v>35</v>
       </c>
-      <c r="H26" t="s">
+      <c r="J26" t="s">
         <v>39</v>
       </c>
-      <c r="I26">
+      <c r="K26">
         <v>592.5</v>
       </c>
-      <c r="J26">
+      <c r="L26">
         <v>557.79999999999995</v>
       </c>
-      <c r="K26">
+      <c r="M26">
         <v>522.29999999999995</v>
       </c>
-      <c r="L26">
+      <c r="N26">
         <v>483</v>
       </c>
-      <c r="M26">
+      <c r="O26">
         <v>445.4</v>
       </c>
-      <c r="N26">
+      <c r="P26">
         <v>414.4</v>
       </c>
-      <c r="O26">
+      <c r="Q26">
         <v>385</v>
       </c>
-      <c r="P26">
+      <c r="R26">
         <v>366.3</v>
       </c>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>32</v>
       </c>
@@ -1918,49 +2102,55 @@
         <v>520.1</v>
       </c>
       <c r="F27" t="s">
+        <v>49</v>
+      </c>
+      <c r="G27" t="s">
+        <v>47</v>
+      </c>
+      <c r="H27" t="s">
         <v>30</v>
       </c>
-      <c r="H27" t="s">
+      <c r="J27" t="s">
         <v>39</v>
       </c>
-      <c r="I27">
+      <c r="K27">
         <v>518.29999999999995</v>
       </c>
-      <c r="J27">
+      <c r="L27">
         <v>485.4</v>
       </c>
-      <c r="K27">
+      <c r="M27">
         <v>457.5</v>
       </c>
-      <c r="L27">
+      <c r="N27">
         <v>429.2</v>
       </c>
-      <c r="M27">
+      <c r="O27">
         <v>403.2</v>
       </c>
-      <c r="N27">
+      <c r="P27">
         <v>376.9</v>
       </c>
-      <c r="O27">
+      <c r="Q27">
         <v>350.2</v>
       </c>
-      <c r="P27">
+      <c r="R27">
         <v>322.39999999999998</v>
       </c>
-      <c r="Q27">
+      <c r="S27">
         <v>295.8</v>
       </c>
-      <c r="R27">
+      <c r="T27">
         <v>269.60000000000002</v>
       </c>
-      <c r="S27">
+      <c r="U27">
         <v>244.2</v>
       </c>
-      <c r="T27">
+      <c r="V27">
         <v>217.7</v>
       </c>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>33</v>
       </c>
@@ -1977,46 +2167,52 @@
         <v>395.7</v>
       </c>
       <c r="F28" t="s">
+        <v>49</v>
+      </c>
+      <c r="G28" t="s">
+        <v>47</v>
+      </c>
+      <c r="H28" t="s">
         <v>34</v>
       </c>
-      <c r="H28" t="s">
+      <c r="J28" t="s">
         <v>40</v>
       </c>
-      <c r="I28">
+      <c r="K28">
         <v>395.7</v>
       </c>
-      <c r="J28">
+      <c r="L28">
         <v>354.4</v>
       </c>
-      <c r="K28">
+      <c r="M28">
         <v>310.5</v>
       </c>
-      <c r="L28">
+      <c r="N28">
         <v>269.39999999999998</v>
       </c>
-      <c r="M28">
+      <c r="O28">
         <v>237.1</v>
       </c>
-      <c r="N28">
+      <c r="P28">
         <v>199.1</v>
       </c>
-      <c r="O28">
+      <c r="Q28">
         <v>172.2</v>
       </c>
-      <c r="P28">
+      <c r="R28">
         <v>150</v>
       </c>
-      <c r="Q28">
+      <c r="S28">
         <v>97</v>
       </c>
-      <c r="R28">
+      <c r="T28">
         <v>74.400000000000006</v>
       </c>
-      <c r="S28">
+      <c r="U28">
         <v>15.4</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>34</v>
       </c>
@@ -2033,25 +2229,31 @@
         <v>385.6</v>
       </c>
       <c r="F29" t="s">
+        <v>49</v>
+      </c>
+      <c r="G29" t="s">
+        <v>47</v>
+      </c>
+      <c r="H29" t="s">
         <v>34</v>
       </c>
-      <c r="H29" t="s">
+      <c r="J29" t="s">
         <v>40</v>
       </c>
-      <c r="I29">
+      <c r="K29">
         <v>385.6</v>
       </c>
-      <c r="J29">
+      <c r="L29">
         <v>368.9</v>
       </c>
-      <c r="K29">
+      <c r="M29">
         <v>343.7</v>
       </c>
-      <c r="L29">
+      <c r="N29">
         <v>318.5</v>
       </c>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>35</v>
       </c>
@@ -2068,61 +2270,67 @@
         <v>540.6</v>
       </c>
       <c r="F30" t="s">
+        <v>49</v>
+      </c>
+      <c r="G30" t="s">
+        <v>46</v>
+      </c>
+      <c r="H30" t="s">
         <v>31</v>
       </c>
-      <c r="H30" t="s">
+      <c r="J30" t="s">
         <v>39</v>
       </c>
-      <c r="I30">
+      <c r="K30">
         <v>538.79999999999995</v>
       </c>
-      <c r="J30">
+      <c r="L30">
         <v>507.2</v>
       </c>
-      <c r="K30">
+      <c r="M30">
         <v>462.9</v>
       </c>
-      <c r="L30">
+      <c r="N30">
         <v>419.3</v>
       </c>
-      <c r="M30">
+      <c r="O30">
         <v>384.8</v>
       </c>
-      <c r="N30">
+      <c r="P30">
         <v>337</v>
       </c>
-      <c r="O30">
+      <c r="Q30">
         <v>304.8</v>
       </c>
-      <c r="P30">
+      <c r="R30">
         <v>264.7</v>
       </c>
-      <c r="Q30">
+      <c r="S30">
         <v>233</v>
       </c>
-      <c r="R30" t="s">
+      <c r="T30" t="s">
         <v>42</v>
       </c>
-      <c r="S30">
+      <c r="U30">
         <v>171</v>
       </c>
-      <c r="T30">
+      <c r="V30">
         <v>137.6</v>
       </c>
-      <c r="U30">
+      <c r="W30">
         <v>112.9</v>
       </c>
-      <c r="V30">
+      <c r="X30">
         <v>70.8</v>
       </c>
-      <c r="W30">
+      <c r="Y30">
         <v>39.4</v>
       </c>
-      <c r="X30">
+      <c r="Z30">
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>36</v>
       </c>
@@ -2139,67 +2347,73 @@
         <v>519.20000000000005</v>
       </c>
       <c r="F31" t="s">
+        <v>49</v>
+      </c>
+      <c r="G31" t="s">
+        <v>47</v>
+      </c>
+      <c r="H31" t="s">
         <v>30</v>
       </c>
-      <c r="H31" t="s">
+      <c r="J31" t="s">
         <v>39</v>
       </c>
-      <c r="I31">
+      <c r="K31">
         <v>517</v>
       </c>
-      <c r="J31">
+      <c r="L31">
         <v>488.6</v>
       </c>
-      <c r="K31">
+      <c r="M31">
         <v>452.7</v>
       </c>
-      <c r="L31">
+      <c r="N31">
         <v>407.3</v>
       </c>
-      <c r="M31">
+      <c r="O31">
         <v>368.1</v>
       </c>
-      <c r="N31">
+      <c r="P31">
         <v>334</v>
       </c>
-      <c r="O31">
+      <c r="Q31">
         <v>302.5</v>
       </c>
-      <c r="P31">
+      <c r="R31">
         <v>282.89999999999998</v>
       </c>
-      <c r="Q31">
+      <c r="S31">
         <v>251.7</v>
       </c>
-      <c r="R31">
+      <c r="T31">
         <v>218.6</v>
       </c>
-      <c r="S31">
+      <c r="U31">
         <v>190.7</v>
       </c>
-      <c r="T31">
+      <c r="V31">
         <v>163.69999999999999</v>
       </c>
-      <c r="U31">
+      <c r="W31">
         <v>140.6</v>
       </c>
-      <c r="V31">
+      <c r="X31">
         <v>117.1</v>
       </c>
-      <c r="W31">
+      <c r="Y31">
         <v>106.4</v>
       </c>
-      <c r="X31">
+      <c r="Z31">
         <v>92.9</v>
       </c>
-      <c r="Y31">
+      <c r="AA31">
         <v>55.5</v>
       </c>
-      <c r="Z31">
+      <c r="AB31">
         <v>26.1</v>
       </c>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>37</v>
       </c>
@@ -2216,25 +2430,31 @@
         <v>444.4</v>
       </c>
       <c r="F32" t="s">
+        <v>51</v>
+      </c>
+      <c r="G32" t="s">
+        <v>48</v>
+      </c>
+      <c r="H32" t="s">
         <v>29</v>
       </c>
-      <c r="H32" t="s">
+      <c r="J32" t="s">
         <v>39</v>
       </c>
-      <c r="I32">
+      <c r="K32">
         <v>444.4</v>
       </c>
-      <c r="J32">
+      <c r="L32">
         <v>315.10000000000002</v>
       </c>
-      <c r="K32">
+      <c r="M32">
         <v>154.9</v>
       </c>
-      <c r="L32">
+      <c r="N32">
         <v>13.3</v>
       </c>
     </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>38</v>
       </c>
@@ -2251,34 +2471,40 @@
         <v>265.8</v>
       </c>
       <c r="F33" t="s">
+        <v>50</v>
+      </c>
+      <c r="G33" t="s">
+        <v>45</v>
+      </c>
+      <c r="H33" t="s">
         <v>25</v>
       </c>
-      <c r="H33" t="s">
+      <c r="J33" t="s">
         <v>39</v>
       </c>
-      <c r="I33">
+      <c r="K33">
         <v>262.8</v>
       </c>
-      <c r="J33">
+      <c r="L33">
         <v>251.1</v>
       </c>
-      <c r="K33">
+      <c r="M33">
         <v>210.5</v>
       </c>
-      <c r="L33">
+      <c r="N33">
         <v>178.4</v>
       </c>
-      <c r="M33">
+      <c r="O33">
         <v>145.30000000000001</v>
       </c>
-      <c r="N33">
+      <c r="P33">
         <v>121.4</v>
       </c>
-      <c r="O33">
+      <c r="Q33">
         <v>94.6</v>
       </c>
     </row>
-    <row r="34" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>39</v>
       </c>
@@ -2295,34 +2521,40 @@
         <v>527.29999999999995</v>
       </c>
       <c r="F34" t="s">
+        <v>49</v>
+      </c>
+      <c r="G34" t="s">
+        <v>47</v>
+      </c>
+      <c r="H34" t="s">
         <v>30</v>
       </c>
-      <c r="H34" t="s">
+      <c r="J34" t="s">
         <v>39</v>
       </c>
-      <c r="I34">
+      <c r="K34">
         <v>525.20000000000005</v>
       </c>
-      <c r="J34">
+      <c r="L34">
         <v>511.1</v>
       </c>
-      <c r="K34">
+      <c r="M34">
         <v>486</v>
       </c>
-      <c r="L34">
+      <c r="N34">
         <v>448.6</v>
       </c>
-      <c r="M34">
+      <c r="O34">
         <v>429.9</v>
       </c>
-      <c r="N34">
+      <c r="P34">
         <v>428.4</v>
       </c>
-      <c r="O34">
+      <c r="Q34">
         <v>421.6</v>
       </c>
     </row>
-    <row r="35" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>40</v>
       </c>
@@ -2339,67 +2571,73 @@
         <v>553.5</v>
       </c>
       <c r="F35" t="s">
+        <v>50</v>
+      </c>
+      <c r="G35" t="s">
+        <v>45</v>
+      </c>
+      <c r="H35" t="s">
         <v>36</v>
       </c>
-      <c r="G35">
+      <c r="I35">
         <v>0.6</v>
       </c>
-      <c r="H35" t="s">
+      <c r="J35" t="s">
         <v>39</v>
       </c>
-      <c r="I35">
+      <c r="K35">
         <v>554.1</v>
       </c>
-      <c r="J35">
+      <c r="L35">
         <v>538.4</v>
       </c>
-      <c r="K35">
+      <c r="M35">
         <v>528</v>
       </c>
-      <c r="L35">
+      <c r="N35">
         <v>521.4</v>
       </c>
-      <c r="M35">
+      <c r="O35">
         <v>516</v>
       </c>
-      <c r="N35">
+      <c r="P35">
         <v>506.3</v>
       </c>
-      <c r="O35" t="s">
+      <c r="Q35" t="s">
         <v>41</v>
       </c>
-      <c r="P35">
+      <c r="R35">
         <v>491.8</v>
       </c>
-      <c r="Q35">
+      <c r="S35">
         <v>486.4</v>
       </c>
-      <c r="R35">
+      <c r="T35">
         <v>480.1</v>
       </c>
-      <c r="S35">
+      <c r="U35">
         <v>475.1</v>
       </c>
-      <c r="T35">
+      <c r="V35">
         <v>464.6</v>
       </c>
-      <c r="U35">
+      <c r="W35">
         <v>453.6</v>
       </c>
-      <c r="V35">
+      <c r="X35">
         <v>448.3</v>
       </c>
-      <c r="W35">
+      <c r="Y35">
         <v>439.1</v>
       </c>
-      <c r="X35">
+      <c r="Z35">
         <v>429.8</v>
       </c>
-      <c r="Y35">
+      <c r="AA35">
         <v>421.4</v>
       </c>
     </row>
-    <row r="36" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>41</v>
       </c>
@@ -2416,46 +2654,52 @@
         <v>338.7</v>
       </c>
       <c r="F36" t="s">
+        <v>51</v>
+      </c>
+      <c r="G36" t="s">
+        <v>48</v>
+      </c>
+      <c r="H36" t="s">
         <v>35</v>
       </c>
-      <c r="H36" t="s">
+      <c r="J36" t="s">
         <v>40</v>
       </c>
-      <c r="I36">
+      <c r="K36">
         <v>338.7</v>
       </c>
-      <c r="J36">
+      <c r="L36">
         <v>332.6</v>
       </c>
-      <c r="K36">
+      <c r="M36">
         <v>275.39999999999998</v>
       </c>
-      <c r="L36">
+      <c r="N36">
         <v>250.5</v>
       </c>
-      <c r="M36">
+      <c r="O36">
         <v>246.4</v>
       </c>
-      <c r="N36">
+      <c r="P36">
         <v>192.8</v>
       </c>
-      <c r="O36">
+      <c r="Q36">
         <v>163.69999999999999</v>
       </c>
-      <c r="P36">
+      <c r="R36">
         <v>140.1</v>
       </c>
-      <c r="Q36">
+      <c r="S36">
         <v>116.4</v>
       </c>
-      <c r="R36">
+      <c r="T36">
         <v>91</v>
       </c>
-      <c r="S36">
+      <c r="U36">
         <v>65.2</v>
       </c>
     </row>
-    <row r="37" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>42</v>
       </c>
@@ -2472,31 +2716,37 @@
         <v>356.2</v>
       </c>
       <c r="F37" t="s">
+        <v>51</v>
+      </c>
+      <c r="G37" t="s">
+        <v>48</v>
+      </c>
+      <c r="H37" t="s">
         <v>35</v>
       </c>
-      <c r="H37" t="s">
+      <c r="J37" t="s">
         <v>39</v>
       </c>
-      <c r="I37">
+      <c r="K37">
         <v>356.2</v>
       </c>
-      <c r="J37">
+      <c r="L37">
         <v>282.8</v>
       </c>
-      <c r="K37">
+      <c r="M37">
         <v>243.3</v>
       </c>
-      <c r="L37">
+      <c r="N37">
         <v>162.30000000000001</v>
       </c>
-      <c r="M37">
+      <c r="O37">
         <v>93.8</v>
       </c>
-      <c r="N37">
+      <c r="P37">
         <v>13.1</v>
       </c>
     </row>
-    <row r="38" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>43</v>
       </c>
@@ -2513,34 +2763,40 @@
         <v>603.1</v>
       </c>
       <c r="F38" t="s">
+        <v>50</v>
+      </c>
+      <c r="G38" t="s">
+        <v>45</v>
+      </c>
+      <c r="H38" t="s">
         <v>36</v>
       </c>
-      <c r="G38">
+      <c r="I38">
         <v>1.7</v>
       </c>
-      <c r="H38" t="s">
+      <c r="J38" t="s">
         <v>39</v>
       </c>
-      <c r="I38">
+      <c r="K38">
         <v>604.79999999999995</v>
       </c>
-      <c r="J38">
+      <c r="L38">
         <v>586.6</v>
       </c>
-      <c r="K38">
+      <c r="M38">
         <v>575</v>
       </c>
-      <c r="L38">
+      <c r="N38">
         <v>562.5</v>
       </c>
-      <c r="M38">
+      <c r="O38">
         <v>547.20000000000005</v>
       </c>
-      <c r="N38">
+      <c r="P38">
         <v>526.1</v>
       </c>
     </row>
-    <row r="39" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>44</v>
       </c>
@@ -2557,34 +2813,40 @@
         <v>568.5</v>
       </c>
       <c r="F39" t="s">
+        <v>50</v>
+      </c>
+      <c r="G39" t="s">
+        <v>45</v>
+      </c>
+      <c r="H39" t="s">
         <v>37</v>
       </c>
-      <c r="H39" t="s">
+      <c r="J39" t="s">
         <v>39</v>
       </c>
-      <c r="I39">
+      <c r="K39">
         <v>568.5</v>
       </c>
-      <c r="J39">
+      <c r="L39">
         <v>556.1</v>
       </c>
-      <c r="K39">
+      <c r="M39">
         <v>531.9</v>
       </c>
-      <c r="L39">
+      <c r="N39">
         <v>518.5</v>
       </c>
-      <c r="M39">
+      <c r="O39">
         <v>511.9</v>
       </c>
-      <c r="N39">
+      <c r="P39">
         <v>504.8</v>
       </c>
-      <c r="O39">
+      <c r="Q39">
         <v>477.4</v>
       </c>
     </row>
-    <row r="40" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>45</v>
       </c>
@@ -2601,46 +2863,52 @@
         <v>362.6</v>
       </c>
       <c r="F40" t="s">
+        <v>51</v>
+      </c>
+      <c r="G40" t="s">
+        <v>48</v>
+      </c>
+      <c r="H40" t="s">
         <v>38</v>
       </c>
-      <c r="H40" t="s">
+      <c r="J40" t="s">
         <v>40</v>
       </c>
-      <c r="I40">
+      <c r="K40">
         <v>363.1</v>
       </c>
-      <c r="J40">
+      <c r="L40">
         <v>329</v>
       </c>
-      <c r="K40">
+      <c r="M40">
         <v>286.2</v>
       </c>
-      <c r="L40">
+      <c r="N40">
         <v>262.5</v>
       </c>
-      <c r="M40">
+      <c r="O40">
         <v>234.4</v>
       </c>
-      <c r="N40">
+      <c r="P40">
         <v>200.4</v>
       </c>
-      <c r="O40">
+      <c r="Q40">
         <v>185.3</v>
       </c>
-      <c r="P40">
+      <c r="R40">
         <v>131.4</v>
       </c>
-      <c r="Q40">
+      <c r="S40">
         <v>54</v>
       </c>
-      <c r="R40">
+      <c r="T40">
         <v>24.9</v>
       </c>
-      <c r="S40">
+      <c r="U40">
         <v>17</v>
       </c>
     </row>
-    <row r="41" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>46</v>
       </c>
@@ -2657,49 +2925,55 @@
         <v>387.7</v>
       </c>
       <c r="F41" t="s">
+        <v>51</v>
+      </c>
+      <c r="G41" t="s">
+        <v>48</v>
+      </c>
+      <c r="H41" t="s">
         <v>35</v>
       </c>
-      <c r="H41" t="s">
+      <c r="J41" t="s">
         <v>39</v>
       </c>
-      <c r="I41">
+      <c r="K41">
         <v>387.7</v>
       </c>
-      <c r="J41">
+      <c r="L41">
         <v>341</v>
       </c>
-      <c r="K41">
+      <c r="M41">
         <v>305.7</v>
       </c>
-      <c r="L41">
+      <c r="N41">
         <v>262.8</v>
       </c>
-      <c r="M41">
+      <c r="O41">
         <v>222.6</v>
       </c>
-      <c r="N41">
+      <c r="P41">
         <v>186.1</v>
       </c>
-      <c r="O41">
+      <c r="Q41">
         <v>157.6</v>
       </c>
-      <c r="P41">
+      <c r="R41">
         <v>119.5</v>
       </c>
-      <c r="Q41">
+      <c r="S41">
         <v>83.5</v>
       </c>
-      <c r="R41">
+      <c r="T41">
         <v>49.8</v>
       </c>
-      <c r="S41">
+      <c r="U41">
         <v>26.8</v>
       </c>
-      <c r="T41">
+      <c r="V41">
         <v>12.9</v>
       </c>
     </row>
-    <row r="42" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>47</v>
       </c>
@@ -2716,46 +2990,52 @@
         <v>356.9</v>
       </c>
       <c r="F42" t="s">
+        <v>51</v>
+      </c>
+      <c r="G42" t="s">
+        <v>48</v>
+      </c>
+      <c r="H42" t="s">
         <v>35</v>
       </c>
-      <c r="H42" t="s">
+      <c r="J42" t="s">
         <v>39</v>
       </c>
-      <c r="I42">
+      <c r="K42">
         <v>356.7</v>
       </c>
-      <c r="J42">
+      <c r="L42">
         <v>339</v>
       </c>
-      <c r="K42">
+      <c r="M42">
         <v>311.2</v>
       </c>
-      <c r="L42">
+      <c r="N42">
         <v>259.60000000000002</v>
       </c>
-      <c r="M42">
+      <c r="O42">
         <v>225.5</v>
       </c>
-      <c r="N42">
+      <c r="P42">
         <v>191</v>
       </c>
-      <c r="O42">
+      <c r="Q42">
         <v>144.80000000000001</v>
       </c>
-      <c r="P42">
+      <c r="R42">
         <v>100.1</v>
       </c>
-      <c r="Q42">
+      <c r="S42">
         <v>53.5</v>
       </c>
-      <c r="R42">
+      <c r="T42">
         <v>30.9</v>
       </c>
-      <c r="S42">
+      <c r="U42">
         <v>12.9</v>
       </c>
     </row>
-    <row r="43" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>48</v>
       </c>
@@ -2772,49 +3052,55 @@
         <v>23</v>
       </c>
       <c r="F43" t="s">
+        <v>51</v>
+      </c>
+      <c r="G43" t="s">
+        <v>48</v>
+      </c>
+      <c r="H43" t="s">
         <v>35</v>
       </c>
-      <c r="H43" t="s">
+      <c r="J43" t="s">
         <v>40</v>
       </c>
-      <c r="I43">
+      <c r="K43">
         <v>362.8</v>
       </c>
-      <c r="J43">
+      <c r="L43">
         <v>322.2</v>
       </c>
-      <c r="K43">
+      <c r="M43">
         <v>284.39999999999998</v>
       </c>
-      <c r="L43">
+      <c r="N43">
         <v>268.3</v>
       </c>
-      <c r="M43">
+      <c r="O43">
         <v>249.2</v>
       </c>
-      <c r="N43">
+      <c r="P43">
         <v>226.9</v>
       </c>
-      <c r="O43">
+      <c r="Q43">
         <v>207</v>
       </c>
-      <c r="P43">
+      <c r="R43">
         <v>188</v>
       </c>
-      <c r="Q43">
+      <c r="S43">
         <v>166.1</v>
       </c>
-      <c r="R43">
+      <c r="T43">
         <v>142.1</v>
       </c>
-      <c r="S43">
+      <c r="U43">
         <v>127.8</v>
       </c>
-      <c r="T43">
+      <c r="V43">
         <v>110</v>
       </c>
     </row>
-    <row r="44" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>49</v>
       </c>
@@ -2831,37 +3117,43 @@
         <v>607.5</v>
       </c>
       <c r="F44" t="s">
+        <v>50</v>
+      </c>
+      <c r="G44" t="s">
+        <v>45</v>
+      </c>
+      <c r="H44" t="s">
         <v>36</v>
       </c>
-      <c r="H44" t="s">
+      <c r="J44" t="s">
         <v>39</v>
       </c>
-      <c r="I44">
+      <c r="K44">
         <v>607.5</v>
       </c>
-      <c r="J44">
+      <c r="L44">
         <v>585</v>
       </c>
-      <c r="K44">
+      <c r="M44">
         <v>567.5</v>
       </c>
-      <c r="L44">
+      <c r="N44">
         <v>541</v>
       </c>
-      <c r="M44">
+      <c r="O44">
         <v>516.29999999999995</v>
       </c>
-      <c r="N44">
+      <c r="P44">
         <v>488.4</v>
       </c>
-      <c r="O44">
+      <c r="Q44">
         <v>467.5</v>
       </c>
-      <c r="P44">
+      <c r="R44">
         <v>442.2</v>
       </c>
     </row>
-    <row r="45" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>50</v>
       </c>
@@ -2878,31 +3170,37 @@
         <v>240.2</v>
       </c>
       <c r="F45" t="s">
+        <v>51</v>
+      </c>
+      <c r="G45" t="s">
+        <v>48</v>
+      </c>
+      <c r="H45" t="s">
         <v>38</v>
       </c>
-      <c r="H45" t="s">
+      <c r="J45" t="s">
         <v>40</v>
       </c>
-      <c r="I45">
+      <c r="K45">
         <v>240.2</v>
       </c>
-      <c r="J45">
+      <c r="L45">
         <v>169.4</v>
       </c>
-      <c r="K45">
+      <c r="M45">
         <v>111.4</v>
       </c>
-      <c r="L45">
+      <c r="N45">
         <v>83.4</v>
       </c>
-      <c r="M45">
+      <c r="O45">
         <v>58.2</v>
       </c>
-      <c r="N45">
+      <c r="P45">
         <v>14.5</v>
       </c>
     </row>
-    <row r="46" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>51</v>
       </c>
@@ -2919,70 +3217,76 @@
         <v>407.9</v>
       </c>
       <c r="F46" t="s">
+        <v>51</v>
+      </c>
+      <c r="G46" t="s">
+        <v>48</v>
+      </c>
+      <c r="H46" t="s">
         <v>35</v>
       </c>
-      <c r="H46" t="s">
+      <c r="J46" t="s">
         <v>40</v>
       </c>
-      <c r="I46">
+      <c r="K46">
         <v>407.9</v>
       </c>
-      <c r="J46">
+      <c r="L46">
         <v>388.9</v>
       </c>
-      <c r="K46">
+      <c r="M46">
         <v>367.9</v>
       </c>
-      <c r="L46">
+      <c r="N46">
         <v>347.7</v>
       </c>
-      <c r="M46">
+      <c r="O46">
         <v>323</v>
       </c>
-      <c r="N46">
+      <c r="P46">
         <v>299.39999999999998</v>
       </c>
-      <c r="O46">
+      <c r="Q46">
         <v>276.7</v>
       </c>
-      <c r="P46">
+      <c r="R46">
         <v>255.3</v>
       </c>
-      <c r="Q46">
+      <c r="S46">
         <v>235.7</v>
       </c>
-      <c r="R46">
+      <c r="T46">
         <v>213.8</v>
       </c>
-      <c r="S46">
+      <c r="U46">
         <v>194.3</v>
       </c>
-      <c r="T46">
+      <c r="V46">
         <v>173.7</v>
       </c>
-      <c r="U46">
+      <c r="W46">
         <v>154.9</v>
       </c>
-      <c r="V46">
+      <c r="X46">
         <v>127.6</v>
       </c>
-      <c r="W46">
+      <c r="Y46">
         <v>109.2</v>
       </c>
-      <c r="X46">
+      <c r="Z46">
         <v>83.4</v>
       </c>
-      <c r="Y46">
+      <c r="AA46">
         <v>59</v>
       </c>
-      <c r="Z46">
+      <c r="AB46">
         <v>48.1</v>
       </c>
-      <c r="AA46">
+      <c r="AC46">
         <v>25.9</v>
       </c>
     </row>
-    <row r="47" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>52</v>
       </c>
@@ -2999,37 +3303,43 @@
         <v>564.70000000000005</v>
       </c>
       <c r="F47" t="s">
+        <v>50</v>
+      </c>
+      <c r="G47" t="s">
+        <v>45</v>
+      </c>
+      <c r="H47" t="s">
         <v>36</v>
       </c>
-      <c r="H47" t="s">
+      <c r="J47" t="s">
         <v>39</v>
       </c>
-      <c r="I47">
+      <c r="K47">
         <v>564.70000000000005</v>
       </c>
-      <c r="J47">
+      <c r="L47">
         <v>547.1</v>
       </c>
-      <c r="K47">
+      <c r="M47">
         <v>533.1</v>
       </c>
-      <c r="L47">
+      <c r="N47">
         <v>516.1</v>
       </c>
-      <c r="M47">
+      <c r="O47">
         <v>505.2</v>
       </c>
-      <c r="N47">
+      <c r="P47">
         <v>489.1</v>
       </c>
-      <c r="O47">
+      <c r="Q47">
         <v>474.9</v>
       </c>
-      <c r="P47">
+      <c r="R47">
         <v>463.4</v>
       </c>
     </row>
-    <row r="48" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>53</v>
       </c>
@@ -3046,40 +3356,46 @@
         <v>365.5</v>
       </c>
       <c r="F48" t="s">
+        <v>51</v>
+      </c>
+      <c r="G48" t="s">
+        <v>48</v>
+      </c>
+      <c r="H48" t="s">
         <v>35</v>
       </c>
-      <c r="H48" t="s">
+      <c r="J48" t="s">
         <v>40</v>
       </c>
-      <c r="I48">
+      <c r="K48">
         <v>365.5</v>
       </c>
-      <c r="J48">
+      <c r="L48">
         <v>320.10000000000002</v>
       </c>
-      <c r="K48">
+      <c r="M48">
         <v>229.9</v>
       </c>
-      <c r="L48">
+      <c r="N48">
         <v>180.6</v>
       </c>
-      <c r="M48">
+      <c r="O48">
         <v>154.30000000000001</v>
       </c>
-      <c r="N48">
+      <c r="P48">
         <v>122.3</v>
       </c>
-      <c r="O48">
+      <c r="Q48">
         <v>91.7</v>
       </c>
-      <c r="P48">
+      <c r="R48">
         <v>64.2</v>
       </c>
-      <c r="Q48">
+      <c r="S48">
         <v>55.2</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>54</v>
       </c>
@@ -3096,40 +3412,46 @@
         <v>567.29999999999995</v>
       </c>
       <c r="F49" t="s">
+        <v>50</v>
+      </c>
+      <c r="G49" t="s">
+        <v>45</v>
+      </c>
+      <c r="H49" t="s">
         <v>36</v>
       </c>
-      <c r="H49" t="s">
+      <c r="J49" t="s">
         <v>39</v>
       </c>
-      <c r="I49">
+      <c r="K49">
         <v>567.29999999999995</v>
       </c>
-      <c r="J49">
+      <c r="L49">
         <v>560.29999999999995</v>
       </c>
-      <c r="K49">
+      <c r="M49">
         <v>540.4</v>
       </c>
-      <c r="L49">
+      <c r="N49">
         <v>531.70000000000005</v>
       </c>
-      <c r="M49">
+      <c r="O49">
         <v>512.9</v>
       </c>
-      <c r="N49">
+      <c r="P49">
         <v>492.9</v>
       </c>
-      <c r="O49">
+      <c r="Q49">
         <v>469.5</v>
       </c>
-      <c r="P49">
+      <c r="R49">
         <v>450.5</v>
       </c>
-      <c r="Q49">
+      <c r="S49">
         <v>327.60000000000002</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>55</v>
       </c>
@@ -3146,49 +3468,55 @@
         <v>353.7</v>
       </c>
       <c r="F50" t="s">
+        <v>51</v>
+      </c>
+      <c r="G50" t="s">
+        <v>48</v>
+      </c>
+      <c r="H50" t="s">
         <v>38</v>
       </c>
-      <c r="H50" t="s">
+      <c r="J50" t="s">
         <v>40</v>
       </c>
-      <c r="I50">
+      <c r="K50">
         <v>353.7</v>
       </c>
-      <c r="J50">
+      <c r="L50">
         <v>305.7</v>
       </c>
-      <c r="K50">
+      <c r="M50">
         <v>272.2</v>
       </c>
-      <c r="L50">
+      <c r="N50">
         <v>230.1</v>
       </c>
-      <c r="M50">
+      <c r="O50">
         <v>207.1</v>
       </c>
-      <c r="N50">
+      <c r="P50">
         <v>172.9</v>
       </c>
-      <c r="O50">
+      <c r="Q50">
         <v>151.6</v>
       </c>
-      <c r="P50">
+      <c r="R50">
         <v>122</v>
       </c>
-      <c r="Q50">
+      <c r="S50">
         <v>104.9</v>
       </c>
-      <c r="R50">
+      <c r="T50">
         <v>79.400000000000006</v>
       </c>
-      <c r="S50">
+      <c r="U50">
         <v>48.1</v>
       </c>
-      <c r="T50">
+      <c r="V50">
         <v>15.1</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>56</v>
       </c>
@@ -3205,46 +3533,52 @@
         <v>577</v>
       </c>
       <c r="F51" t="s">
+        <v>50</v>
+      </c>
+      <c r="G51" t="s">
+        <v>45</v>
+      </c>
+      <c r="H51" t="s">
         <v>36</v>
       </c>
-      <c r="H51" t="s">
+      <c r="J51" t="s">
         <v>39</v>
       </c>
-      <c r="I51">
+      <c r="K51">
         <v>577</v>
       </c>
-      <c r="J51">
+      <c r="L51">
         <v>563</v>
       </c>
-      <c r="K51">
+      <c r="M51">
         <v>528.70000000000005</v>
       </c>
-      <c r="L51">
+      <c r="N51">
         <v>498.3</v>
       </c>
-      <c r="M51">
+      <c r="O51">
         <v>472.3</v>
       </c>
-      <c r="N51">
+      <c r="P51">
         <v>446</v>
       </c>
-      <c r="O51">
+      <c r="Q51">
         <v>420.4</v>
       </c>
-      <c r="P51">
+      <c r="R51">
         <v>401.7</v>
       </c>
-      <c r="Q51">
+      <c r="S51">
         <v>377.7</v>
       </c>
-      <c r="R51">
+      <c r="T51">
         <v>356.4</v>
       </c>
-      <c r="S51">
+      <c r="U51">
         <v>329</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>57</v>
       </c>
@@ -3261,43 +3595,49 @@
         <v>271.2</v>
       </c>
       <c r="F52" t="s">
+        <v>51</v>
+      </c>
+      <c r="G52" t="s">
+        <v>48</v>
+      </c>
+      <c r="H52" t="s">
         <v>38</v>
       </c>
-      <c r="H52" t="s">
+      <c r="J52" t="s">
         <v>40</v>
       </c>
-      <c r="I52">
+      <c r="K52">
         <v>271.2</v>
       </c>
-      <c r="J52">
+      <c r="L52">
         <v>253.8</v>
       </c>
-      <c r="K52">
+      <c r="M52">
         <v>230.3</v>
       </c>
-      <c r="L52">
+      <c r="N52">
         <v>211.6</v>
       </c>
-      <c r="M52">
+      <c r="O52">
         <v>189.3</v>
       </c>
-      <c r="N52">
+      <c r="P52">
         <v>173</v>
       </c>
-      <c r="O52">
+      <c r="Q52">
         <v>151.80000000000001</v>
       </c>
-      <c r="P52">
+      <c r="R52">
         <v>134.5</v>
       </c>
-      <c r="Q52">
+      <c r="S52">
         <v>113.1</v>
       </c>
-      <c r="R52">
+      <c r="T52">
         <v>93.6</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>58</v>
       </c>
@@ -3314,43 +3654,49 @@
         <v>212.4</v>
       </c>
       <c r="F53" t="s">
+        <v>51</v>
+      </c>
+      <c r="G53" t="s">
+        <v>48</v>
+      </c>
+      <c r="H53" t="s">
         <v>35</v>
       </c>
-      <c r="H53" t="s">
+      <c r="J53" t="s">
         <v>40</v>
       </c>
-      <c r="I53">
+      <c r="K53">
         <v>212.4</v>
       </c>
-      <c r="J53">
+      <c r="L53">
         <v>201.4</v>
       </c>
-      <c r="K53">
+      <c r="M53">
         <v>189.8</v>
       </c>
-      <c r="L53">
+      <c r="N53">
         <v>180.3</v>
       </c>
-      <c r="M53">
+      <c r="O53">
         <v>166.7</v>
       </c>
-      <c r="N53">
+      <c r="P53">
         <v>159.69999999999999</v>
       </c>
-      <c r="O53">
+      <c r="Q53">
         <v>146.1</v>
       </c>
-      <c r="P53">
+      <c r="R53">
         <v>135.4</v>
       </c>
-      <c r="Q53">
+      <c r="S53">
         <v>123.6</v>
       </c>
-      <c r="R53">
+      <c r="T53">
         <v>112.5</v>
       </c>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>59</v>
       </c>
@@ -3367,31 +3713,37 @@
         <v>133.9</v>
       </c>
       <c r="F54" t="s">
+        <v>51</v>
+      </c>
+      <c r="G54" t="s">
+        <v>48</v>
+      </c>
+      <c r="H54" t="s">
         <v>35</v>
       </c>
-      <c r="H54" t="s">
+      <c r="J54" t="s">
         <v>40</v>
       </c>
-      <c r="I54">
+      <c r="K54">
         <v>133.9</v>
       </c>
-      <c r="J54">
+      <c r="L54">
         <v>109.1</v>
       </c>
-      <c r="K54">
+      <c r="M54">
         <v>64.099999999999994</v>
       </c>
-      <c r="L54">
+      <c r="N54">
         <v>39.1</v>
       </c>
-      <c r="M54">
+      <c r="O54">
         <v>38.299999999999997</v>
       </c>
-      <c r="N54">
+      <c r="P54">
         <v>15.8</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>60</v>
       </c>
@@ -3408,31 +3760,37 @@
         <v>297.10000000000002</v>
       </c>
       <c r="F55" t="s">
+        <v>51</v>
+      </c>
+      <c r="G55" t="s">
+        <v>48</v>
+      </c>
+      <c r="H55" t="s">
         <v>35</v>
       </c>
-      <c r="H55" t="s">
+      <c r="J55" t="s">
         <v>39</v>
       </c>
-      <c r="I55">
+      <c r="K55">
         <v>297.10000000000002</v>
       </c>
-      <c r="J55">
+      <c r="L55">
         <v>226.3</v>
       </c>
-      <c r="K55">
+      <c r="M55">
         <v>147.4</v>
       </c>
-      <c r="L55">
+      <c r="N55">
         <v>100.9</v>
       </c>
-      <c r="M55">
+      <c r="O55">
         <v>40.9</v>
       </c>
-      <c r="N55">
+      <c r="P55">
         <v>12.9</v>
       </c>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>61</v>
       </c>
@@ -3449,43 +3807,49 @@
         <v>316.3</v>
       </c>
       <c r="F56" t="s">
+        <v>51</v>
+      </c>
+      <c r="G56" t="s">
+        <v>48</v>
+      </c>
+      <c r="H56" t="s">
         <v>35</v>
       </c>
-      <c r="H56" t="s">
+      <c r="J56" t="s">
         <v>39</v>
       </c>
-      <c r="I56">
+      <c r="K56">
         <v>316.3</v>
       </c>
-      <c r="J56">
+      <c r="L56">
         <v>299.89999999999998</v>
       </c>
-      <c r="K56">
+      <c r="M56">
         <v>274.10000000000002</v>
       </c>
-      <c r="L56">
+      <c r="N56">
         <v>259.89999999999998</v>
       </c>
-      <c r="M56">
+      <c r="O56">
         <v>236.8</v>
       </c>
-      <c r="N56">
+      <c r="P56">
         <v>212.7</v>
       </c>
-      <c r="O56">
+      <c r="Q56">
         <v>193.2</v>
       </c>
-      <c r="P56">
+      <c r="R56">
         <v>180.1</v>
       </c>
-      <c r="Q56">
+      <c r="S56">
         <v>163</v>
       </c>
-      <c r="R56">
+      <c r="T56">
         <v>121.8</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>62</v>
       </c>
@@ -3502,33 +3866,39 @@
         <v>336.8</v>
       </c>
       <c r="F57" t="s">
+        <v>51</v>
+      </c>
+      <c r="G57" t="s">
+        <v>48</v>
+      </c>
+      <c r="H57" t="s">
         <v>35</v>
       </c>
-      <c r="H57" t="s">
+      <c r="J57" t="s">
         <v>39</v>
       </c>
-      <c r="I57">
+      <c r="K57">
         <v>336.8</v>
       </c>
-      <c r="J57">
+      <c r="L57">
         <v>300.89999999999998</v>
       </c>
-      <c r="K57">
+      <c r="M57">
         <v>278</v>
       </c>
-      <c r="L57">
+      <c r="N57">
         <v>248.9</v>
       </c>
-      <c r="M57">
+      <c r="O57">
         <v>213.7</v>
       </c>
-      <c r="N57">
+      <c r="P57">
         <v>183.9</v>
       </c>
-      <c r="O57">
+      <c r="Q57">
         <v>150</v>
       </c>
-      <c r="P57">
+      <c r="R57">
         <v>123.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
time to give it to linear reg
</commit_message>
<xml_diff>
--- a/labeled/Hydrocare_ffinal.xlsx
+++ b/labeled/Hydrocare_ffinal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alireza.mohammadshafie/Documents/hydrocare/labeled/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D96F8C8-9C03-2046-8671-2BFBED2F5D34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C702EB-8383-5D45-BC65-A07EB911B6AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="48">
   <si>
     <t>ID</t>
   </si>
@@ -77,18 +77,6 @@
   </si>
   <si>
     <t>Female</t>
-  </si>
-  <si>
-    <t>male</t>
-  </si>
-  <si>
-    <t>female</t>
-  </si>
-  <si>
-    <t>fEMALE</t>
-  </si>
-  <si>
-    <t>famale</t>
   </si>
   <si>
     <t>362.8 with straw</t>
@@ -571,10 +559,10 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>5</v>
@@ -660,16 +648,16 @@
         <v>540.4</v>
       </c>
       <c r="F2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K2">
         <v>538.6</v>
@@ -710,16 +698,16 @@
         <v>272.60000000000002</v>
       </c>
       <c r="F3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J3" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K3">
         <v>272.60000000000002</v>
@@ -763,16 +751,16 @@
         <v>542.6</v>
       </c>
       <c r="F4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="J4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K4">
         <v>540.6</v>
@@ -813,16 +801,16 @@
         <v>542.9</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="J5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K5">
         <v>540.79999999999995</v>
@@ -866,16 +854,16 @@
         <v>521.70000000000005</v>
       </c>
       <c r="F6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="J6" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K6">
         <v>518.79999999999995</v>
@@ -922,16 +910,16 @@
         <v>228.4</v>
       </c>
       <c r="F7" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="J7" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K7">
         <v>228.4</v>
@@ -978,16 +966,16 @@
         <v>519.4</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H8" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="J8" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K8">
         <v>519.20000000000005</v>
@@ -1043,16 +1031,16 @@
         <v>521.20000000000005</v>
       </c>
       <c r="F9" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H9" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J9" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K9">
         <v>519.29999999999995</v>
@@ -1111,16 +1099,16 @@
         <v>515.9</v>
       </c>
       <c r="F10" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G10" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H10" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="J10" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K10">
         <v>515.20000000000005</v>
@@ -1173,16 +1161,16 @@
         <v>547.20000000000005</v>
       </c>
       <c r="F11" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G11" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H11" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="J11" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K11">
         <v>545.70000000000005</v>
@@ -1226,16 +1214,16 @@
         <v>295.10000000000002</v>
       </c>
       <c r="F12" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G12" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H12" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J12" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K12">
         <v>289.5</v>
@@ -1300,16 +1288,16 @@
         <v>542</v>
       </c>
       <c r="F13" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G13" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H13" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J13" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K13">
         <v>539.79999999999995</v>
@@ -1347,7 +1335,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C14">
         <v>19.8</v>
@@ -1359,16 +1347,16 @@
         <v>543.29999999999995</v>
       </c>
       <c r="F14" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G14" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H14" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J14" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K14">
         <v>541.6</v>
@@ -1421,7 +1409,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C15">
         <v>19.8</v>
@@ -1433,16 +1421,16 @@
         <v>518</v>
       </c>
       <c r="F15" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G15" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H15" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J15" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K15">
         <v>472.9</v>
@@ -1465,7 +1453,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C16">
         <v>7.7</v>
@@ -1474,16 +1462,16 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G16" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H16" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="J16" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K16">
         <v>485.4</v>
@@ -1518,7 +1506,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C17">
         <v>10.9</v>
@@ -1530,16 +1518,16 @@
         <v>262.7</v>
       </c>
       <c r="F17" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G17" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H17" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="J17" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K17">
         <v>262.60000000000002</v>
@@ -1571,7 +1559,7 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C18">
         <v>10.9</v>
@@ -1583,16 +1571,16 @@
         <v>280.3</v>
       </c>
       <c r="F18" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G18" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H18" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J18" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K18">
         <v>292.2</v>
@@ -1636,7 +1624,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C19">
         <v>19.8</v>
@@ -1645,16 +1633,16 @@
         <v>1.05</v>
       </c>
       <c r="F19" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G19" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H19" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J19" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K19">
         <v>544.70000000000005</v>
@@ -1689,7 +1677,7 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C20">
         <v>19.8</v>
@@ -1701,16 +1689,16 @@
         <v>518.9</v>
       </c>
       <c r="F20" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G20" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H20" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J20" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K20">
         <v>517</v>
@@ -1751,7 +1739,7 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C21">
         <v>19.8</v>
@@ -1763,16 +1751,16 @@
         <v>523.70000000000005</v>
       </c>
       <c r="F21" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G21" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H21" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J21" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K21">
         <v>521.5</v>
@@ -1798,7 +1786,7 @@
         <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C22">
         <v>7.7</v>
@@ -1810,16 +1798,16 @@
         <v>516.1</v>
       </c>
       <c r="F22" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G22" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H22" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="J22" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K22">
         <v>515.4</v>
@@ -1845,7 +1833,7 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C23">
         <v>12.7</v>
@@ -1857,16 +1845,16 @@
         <v>201.8</v>
       </c>
       <c r="F23" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G23" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H23" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="J23" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K23">
         <v>201.8</v>
@@ -1904,7 +1892,7 @@
         <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C24">
         <v>12.7</v>
@@ -1916,16 +1904,16 @@
         <v>330.5</v>
       </c>
       <c r="F24" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G24" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H24" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="J24" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K24">
         <v>331.2</v>
@@ -1963,7 +1951,7 @@
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C25">
         <v>19.8</v>
@@ -1975,16 +1963,16 @@
         <v>548.79999999999995</v>
       </c>
       <c r="F25" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G25" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H25" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J25" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K25">
         <v>546.6</v>
@@ -2037,7 +2025,7 @@
         <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C26">
         <v>12.7</v>
@@ -2049,16 +2037,16 @@
         <v>592.5</v>
       </c>
       <c r="F26" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G26" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H26" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J26" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K26">
         <v>592.5</v>
@@ -2090,7 +2078,7 @@
         <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C27">
         <v>19.8</v>
@@ -2102,16 +2090,16 @@
         <v>520.1</v>
       </c>
       <c r="F27" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G27" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H27" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J27" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K27">
         <v>518.29999999999995</v>
@@ -2155,7 +2143,7 @@
         <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C28">
         <v>12.7</v>
@@ -2167,16 +2155,16 @@
         <v>395.7</v>
       </c>
       <c r="F28" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G28" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H28" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="J28" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K28">
         <v>395.7</v>
@@ -2217,7 +2205,7 @@
         <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C29">
         <v>12.7</v>
@@ -2229,16 +2217,16 @@
         <v>385.6</v>
       </c>
       <c r="F29" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G29" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H29" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="J29" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K29">
         <v>385.6</v>
@@ -2258,7 +2246,7 @@
         <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C30">
         <v>19.8</v>
@@ -2270,16 +2258,16 @@
         <v>540.6</v>
       </c>
       <c r="F30" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G30" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H30" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="J30" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K30">
         <v>538.79999999999995</v>
@@ -2309,7 +2297,7 @@
         <v>233</v>
       </c>
       <c r="T30" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="U30">
         <v>171</v>
@@ -2335,7 +2323,7 @@
         <v>36</v>
       </c>
       <c r="B31" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C31">
         <v>19.8</v>
@@ -2347,16 +2335,16 @@
         <v>519.20000000000005</v>
       </c>
       <c r="F31" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G31" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H31" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J31" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K31">
         <v>517</v>
@@ -2418,7 +2406,7 @@
         <v>37</v>
       </c>
       <c r="B32" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C32">
         <v>7.7</v>
@@ -2430,16 +2418,16 @@
         <v>444.4</v>
       </c>
       <c r="F32" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G32" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H32" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="J32" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K32">
         <v>444.4</v>
@@ -2459,7 +2447,7 @@
         <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C33">
         <v>10.9</v>
@@ -2471,16 +2459,16 @@
         <v>265.8</v>
       </c>
       <c r="F33" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G33" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H33" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J33" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K33">
         <v>262.8</v>
@@ -2509,7 +2497,7 @@
         <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C34">
         <v>19.8</v>
@@ -2521,16 +2509,16 @@
         <v>527.29999999999995</v>
       </c>
       <c r="F34" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G34" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H34" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J34" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K34">
         <v>525.20000000000005</v>
@@ -2559,7 +2547,7 @@
         <v>40</v>
       </c>
       <c r="B35" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C35">
         <v>359</v>
@@ -2571,19 +2559,19 @@
         <v>553.5</v>
       </c>
       <c r="F35" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G35" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H35" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="I35">
         <v>0.6</v>
       </c>
       <c r="J35" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K35">
         <v>554.1</v>
@@ -2604,7 +2592,7 @@
         <v>506.3</v>
       </c>
       <c r="Q35" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="R35">
         <v>491.8</v>
@@ -2642,7 +2630,7 @@
         <v>41</v>
       </c>
       <c r="B36" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C36">
         <v>12.7</v>
@@ -2654,16 +2642,16 @@
         <v>338.7</v>
       </c>
       <c r="F36" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G36" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H36" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J36" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K36">
         <v>338.7</v>
@@ -2704,7 +2692,7 @@
         <v>42</v>
       </c>
       <c r="B37" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C37">
         <v>12.7</v>
@@ -2716,16 +2704,16 @@
         <v>356.2</v>
       </c>
       <c r="F37" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G37" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H37" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J37" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K37">
         <v>356.2</v>
@@ -2751,7 +2739,7 @@
         <v>43</v>
       </c>
       <c r="B38" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C38">
         <v>359</v>
@@ -2763,19 +2751,19 @@
         <v>603.1</v>
       </c>
       <c r="F38" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G38" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H38" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="I38">
         <v>1.7</v>
       </c>
       <c r="J38" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K38">
         <v>604.79999999999995</v>
@@ -2801,7 +2789,7 @@
         <v>44</v>
       </c>
       <c r="B39" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C39">
         <v>359</v>
@@ -2813,16 +2801,16 @@
         <v>568.5</v>
       </c>
       <c r="F39" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G39" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H39" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="J39" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K39">
         <v>568.5</v>
@@ -2851,7 +2839,7 @@
         <v>45</v>
       </c>
       <c r="B40" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C40">
         <v>12.7</v>
@@ -2863,16 +2851,16 @@
         <v>362.6</v>
       </c>
       <c r="F40" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G40" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H40" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="J40" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K40">
         <v>363.1</v>
@@ -2913,7 +2901,7 @@
         <v>46</v>
       </c>
       <c r="B41" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C41">
         <v>12.7</v>
@@ -2925,16 +2913,16 @@
         <v>387.7</v>
       </c>
       <c r="F41" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G41" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H41" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J41" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K41">
         <v>387.7</v>
@@ -2978,7 +2966,7 @@
         <v>47</v>
       </c>
       <c r="B42" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C42">
         <v>12.7</v>
@@ -2990,16 +2978,16 @@
         <v>356.9</v>
       </c>
       <c r="F42" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G42" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H42" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J42" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K42">
         <v>356.7</v>
@@ -3040,7 +3028,7 @@
         <v>48</v>
       </c>
       <c r="B43" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C43">
         <v>12.7</v>
@@ -3049,19 +3037,19 @@
         <v>1</v>
       </c>
       <c r="E43" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F43" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G43" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H43" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J43" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K43">
         <v>362.8</v>
@@ -3105,7 +3093,7 @@
         <v>49</v>
       </c>
       <c r="B44" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C44">
         <v>359</v>
@@ -3117,16 +3105,16 @@
         <v>607.5</v>
       </c>
       <c r="F44" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G44" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H44" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="J44" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K44">
         <v>607.5</v>
@@ -3158,7 +3146,7 @@
         <v>50</v>
       </c>
       <c r="B45" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C45">
         <v>12.7</v>
@@ -3170,16 +3158,16 @@
         <v>240.2</v>
       </c>
       <c r="F45" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G45" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H45" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="J45" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K45">
         <v>240.2</v>
@@ -3205,7 +3193,7 @@
         <v>51</v>
       </c>
       <c r="B46" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C46">
         <v>12.7</v>
@@ -3217,16 +3205,16 @@
         <v>407.9</v>
       </c>
       <c r="F46" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G46" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H46" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J46" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K46">
         <v>407.9</v>
@@ -3291,7 +3279,7 @@
         <v>52</v>
       </c>
       <c r="B47" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C47">
         <v>359</v>
@@ -3303,16 +3291,16 @@
         <v>564.70000000000005</v>
       </c>
       <c r="F47" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G47" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H47" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="J47" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K47">
         <v>564.70000000000005</v>
@@ -3344,7 +3332,7 @@
         <v>53</v>
       </c>
       <c r="B48" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C48">
         <v>12.7</v>
@@ -3356,16 +3344,16 @@
         <v>365.5</v>
       </c>
       <c r="F48" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G48" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H48" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J48" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K48">
         <v>365.5</v>
@@ -3400,7 +3388,7 @@
         <v>54</v>
       </c>
       <c r="B49" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C49">
         <v>359</v>
@@ -3412,16 +3400,16 @@
         <v>567.29999999999995</v>
       </c>
       <c r="F49" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G49" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H49" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="J49" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K49">
         <v>567.29999999999995</v>
@@ -3456,7 +3444,7 @@
         <v>55</v>
       </c>
       <c r="B50" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C50">
         <v>12.7</v>
@@ -3468,16 +3456,16 @@
         <v>353.7</v>
       </c>
       <c r="F50" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G50" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H50" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="J50" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K50">
         <v>353.7</v>
@@ -3521,7 +3509,7 @@
         <v>56</v>
       </c>
       <c r="B51" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C51">
         <v>359</v>
@@ -3533,16 +3521,16 @@
         <v>577</v>
       </c>
       <c r="F51" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G51" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H51" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="J51" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K51">
         <v>577</v>
@@ -3583,7 +3571,7 @@
         <v>57</v>
       </c>
       <c r="B52" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C52">
         <v>12.7</v>
@@ -3595,16 +3583,16 @@
         <v>271.2</v>
       </c>
       <c r="F52" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G52" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H52" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="J52" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K52">
         <v>271.2</v>
@@ -3642,7 +3630,7 @@
         <v>58</v>
       </c>
       <c r="B53" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C53">
         <v>12.7</v>
@@ -3654,16 +3642,16 @@
         <v>212.4</v>
       </c>
       <c r="F53" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G53" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H53" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J53" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K53">
         <v>212.4</v>
@@ -3701,7 +3689,7 @@
         <v>59</v>
       </c>
       <c r="B54" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C54">
         <v>12.7</v>
@@ -3713,16 +3701,16 @@
         <v>133.9</v>
       </c>
       <c r="F54" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G54" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H54" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J54" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K54">
         <v>133.9</v>
@@ -3748,7 +3736,7 @@
         <v>60</v>
       </c>
       <c r="B55" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C55">
         <v>12.7</v>
@@ -3760,16 +3748,16 @@
         <v>297.10000000000002</v>
       </c>
       <c r="F55" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G55" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H55" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J55" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K55">
         <v>297.10000000000002</v>
@@ -3795,7 +3783,7 @@
         <v>61</v>
       </c>
       <c r="B56" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C56">
         <v>12.7</v>
@@ -3807,16 +3795,16 @@
         <v>316.3</v>
       </c>
       <c r="F56" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G56" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H56" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J56" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K56">
         <v>316.3</v>
@@ -3854,7 +3842,7 @@
         <v>62</v>
       </c>
       <c r="B57" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C57">
         <v>12.7</v>
@@ -3866,16 +3854,16 @@
         <v>336.8</v>
       </c>
       <c r="F57" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G57" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H57" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="J57" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K57">
         <v>336.8</v>

</xml_diff>